<commit_message>
docs: update master plan, syllabi, quiz guide and rebuild log
</commit_message>
<xml_diff>
--- a/IUEA_Teaching_Plan/IUEA_ML_Semester1_Master_Teaching_Plan.xlsx
+++ b/IUEA_Teaching_Plan/IUEA_ML_Semester1_Master_Teaching_Plan.xlsx
@@ -14090,7 +14090,7 @@
       </c>
       <c r="E22" s="47" t="inlineStr">
         <is>
-          <t>Best 4 of 6 weekly (3 of 5 where W6 is waived) plus both blocks; 50 marks (45)</t>
+          <t>Best 3 of 5 weekly (Week 6 waived) plus both blocks; 45 marks</t>
         </is>
       </c>
       <c r="F22" s="47" t="n"/>
@@ -14116,7 +14116,7 @@
       </c>
       <c r="E23" s="47" t="inlineStr">
         <is>
-          <t>Best 4 of 6 weekly (3 of 5) plus both blocks; 180 marks (160)</t>
+          <t>Best 3 of 5 weekly (Week 6 waived) plus both blocks; 160 marks</t>
         </is>
       </c>
       <c r="F23" s="47" t="n"/>

</xml_diff>

<commit_message>
docs: update master plan, syllabi, guides and rebuild log
</commit_message>
<xml_diff>
--- a/IUEA_Teaching_Plan/IUEA_ML_Semester1_Master_Teaching_Plan.xlsx
+++ b/IUEA_Teaching_Plan/IUEA_ML_Semester1_Master_Teaching_Plan.xlsx
@@ -740,6 +740,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="19.5" customHeight="1" s="36">
       <c r="A4" s="39" t="inlineStr">
         <is>
@@ -795,6 +796,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="19.5" customHeight="1" s="36">
       <c r="A10" s="39" t="inlineStr">
         <is>
@@ -942,6 +944,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17" ht="61.5" customHeight="1" s="36">
       <c r="A17" s="45" t="inlineStr">
         <is>
@@ -949,6 +952,7 @@
         </is>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="19.5" customHeight="1" s="36">
       <c r="A19" s="39" t="inlineStr">
         <is>
@@ -1084,6 +1088,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="19.5" customHeight="1" s="36">
       <c r="A25" s="39" t="inlineStr">
         <is>
@@ -1151,6 +1156,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="19.5" customHeight="1" s="36">
       <c r="A32" s="39" t="inlineStr">
         <is>
@@ -1290,6 +1296,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="45.75" customHeight="1" s="36">
       <c r="A45" s="50" t="inlineStr">
         <is>
@@ -1367,6 +1374,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -1944,6 +1952,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28" ht="39.75" customHeight="1" s="36">
       <c r="A28" s="56" t="inlineStr">
         <is>
@@ -1996,6 +2005,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -2836,6 +2846,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25" ht="43.5" customHeight="1" s="36">
       <c r="A25" s="56" t="inlineStr">
         <is>
@@ -2887,6 +2898,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -3111,6 +3123,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12" ht="45.75" customHeight="1" s="36">
       <c r="A12" s="56" t="inlineStr">
         <is>
@@ -3161,6 +3174,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -3444,6 +3458,7 @@
         </is>
       </c>
     </row>
+    <row r="15"/>
     <row r="16" ht="31.5" customHeight="1" s="36">
       <c r="A16" s="45" t="inlineStr">
         <is>
@@ -3451,6 +3466,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18" ht="61.5" customHeight="1" s="36">
       <c r="A18" s="41" t="inlineStr">
         <is>
@@ -3503,6 +3519,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -3622,7 +3639,7 @@
       </c>
       <c r="E7" s="54" t="inlineStr">
         <is>
-          <t>Confirm seats, working sockets, concurrent Colab access and accessible lab capacity with the Faculty. Stage the cohort notebooks and datasets locally for all three cohorts. Pre-provision the offline environment for connectivity failures and the Week 7/14 tests. Confirm any additional test sittings and invigilation before release.</t>
+          <t>Confirm seats, working sockets, concurrent Colab access and accessible lab capacity with the Faculty. Stage the cohort notebooks and datasets locally for all three cohorts. Pre-provision the offline environment for connectivity failures in teaching sessions. Confirm any additional test sittings and invigilation before release.</t>
         </is>
       </c>
       <c r="F7" s="54" t="inlineStr">
@@ -3750,7 +3767,7 @@
       </c>
       <c r="E11" s="54" t="inlineStr">
         <is>
-          <t>Keep the issued notebooks, datasets and task sheets available locally. Practical tests use the prepared offline environment; Colab teaching and Google Forms still require connectivity. Agree a documented interruption, collection and rescheduling procedure with the Faculty before the tests.</t>
+          <t>Keep the issued notebooks, datasets and task sheets available locally. The practical tests run in Colab and the submission form, so they need connectivity too. Agree a documented interruption, collection and rescheduling procedure with the Faculty before the tests.</t>
         </is>
       </c>
       <c r="F11" s="54" t="inlineStr">
@@ -3846,7 +3863,7 @@
       </c>
       <c r="E14" s="52" t="inlineStr">
         <is>
-          <t>Use matched dataset variants and suitable seating. Offline delivery reduces network communication but does not itself disable local AI tools; maintain invigilated no-AI conditions under Faculty arrangements. Request adequate invigilation for each sitting. Collect the notebook and the individual typed Part B evidence with invigilator-controlled timestamps.</t>
+          <t>Use matched dataset variants and suitable seating. The tests run in Colab, which cannot block AI tools; rely on matched variants, hidden-data grading and the understanding check. Request adequate invigilation for each sitting. Collect the notebook snapshot and the form confirmation with server timestamps.</t>
         </is>
       </c>
       <c r="F14" s="52" t="inlineStr">
@@ -4006,7 +4023,7 @@
       </c>
       <c r="E19" s="52" t="inlineStr">
         <is>
-          <t>Require an AI-use declaration for coursework. Both practical tests prohibit AI and use invigilated offline arrangements; offline mode alone does not enforce that rule. Individual typed defence and Part B answers assess submitted explanations. Do not infer misconduct from writing style or an automated AI detector.</t>
+          <t>Require an AI-use declaration for coursework. Both practical tests prohibit AI. Test 1 is a take-home test with an understanding check and Test 2 follows the invigilator's rules. Only code a student can explain earns marks, because the grader re-runs it on other data. Do not infer misconduct from writing style or an automated AI detector.</t>
         </is>
       </c>
       <c r="F19" s="52" t="inlineStr">
@@ -4154,6 +4171,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -4452,7 +4470,7 @@
       </c>
       <c r="H11" s="54" t="inlineStr">
         <is>
-          <t>Practical Test 1 - Data Investigation (individual, offline, 2h25).</t>
+          <t>Practical Test 1 - Data Investigation (individual, timed Colab practical, 3 hours).</t>
         </is>
       </c>
     </row>
@@ -4708,7 +4726,7 @@
       </c>
       <c r="H18" s="54" t="inlineStr">
         <is>
-          <t>Practical Test 2 - End-to-End Engineering ML (individual, offline, 2h25).</t>
+          <t>Practical Test 2 - End-to-End Engineering ML (individual, timed Colab practical, 3 hours).</t>
         </is>
       </c>
     </row>
@@ -4752,6 +4770,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="15" customHeight="1" s="36">
       <c r="A21" s="40" t="inlineStr">
         <is>
@@ -4819,6 +4838,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="39.75" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -5510,25 +5530,23 @@
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 1 - Data Investigation (individual, offline)</t>
+          <t>PRACTICAL TEST 1 - Data Investigation (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="D11" s="54" t="inlineStr">
         <is>
-          <t>• Independently investigate an unfamiliar engineering dataset under time pressure.
-• Profile, clean and justify, without a prescribed method.
-• Answer stated questions with evidence and correct units.
-• Produce charts that answer questions.
-• Draw an engineering conclusion and state what further data would be needed.
-• Explain their own reasoning in typed offline responses, without executing code or using AI.</t>
+          <t>• Read, inspect and clean an unfamiliar engineering dataset without a prescribed method, and check the result with charts.
+• Calculate summary statistics and group means with pandas and report them accurately.
+• Write a function that works on any table, and a loop with conditions.
+• Explain their own submitted code when asked, without AI or another person's help.</t>
         </is>
       </c>
       <c r="E11" s="54" t="inlineStr">
         <is>
-          <t>• 0:00-0:15  Seating, machine allocation, dataset variant distribution, rules read aloud, offline mode confirmed.
-• 0:15-2:15  TEST, PART A (practical, 2 hours). Individual. An unfamiliar dataset from the cohort's domain plus a task sheet: load and profile; identify and handle defects with a written justification for each; answer three stated engineering questions with evidence; produce three charts, each captioned with the question it answers; list five findings; make one engineering recommendation.
-• 2:15-2:40  TEST, PART B (written reasoning, 25 minutes, typed offline responses only; no code execution). Four short questions on their own submission: why that cleaning decision, what the chart does not show, what would change the conclusion, and what data is missing.
-• 2:40-3:00  Collection, checksum of submissions, immediate structural check, dismissal.</t>
+          <t>• 0:00-0:10  Entry link, private notebook and CSV, rules read aloud, identity cell checked.
+• 0:10-2:25  CODING (135 minutes). Individual, in Colab. Eight coded tasks: read and inspect the file, a chart before cleaning, cleaning, a chart after cleaning, statistics, grouping, one function, and a loop with conditions.
+• 2:25-2:40  CHECKING (15 minutes). Restart the session and Run all.
+• 2:40-3:00  FINAL SAVE AND SUBMISSION (20 minutes). Submit test button, generated form link, confirmation.</t>
         </is>
       </c>
       <c r="F11" s="54" t="inlineStr">
@@ -5539,14 +5557,14 @@
       </c>
       <c r="G11" s="54" t="inlineStr">
         <is>
-          <t>• Permitted: Python, VS Code or Jupyter, pandas, NumPy, matplotlib, seaborn, and an OFFLINE documentation bundle.
-• Prohibited: internet access, AI assistants, messaging and shared drives. Use the invigilated offline lab and approved-materials checks; offline access alone does not prevent a local AI assistant.
+          <t>• Permitted: Colab, pandas, matplotlib, ordinary Python, and your lecture slides, revision guide, cheatsheet and personal course notes.
+• Prohibited: AI tools, help from another person and copied work. Colab cannot block an AI assistant, so the rule rests on the declaration, hidden-data grading and an understanding check in which a student may be asked to explain or change their own code.
 • Rationale published to students in Week 6: AI is permitted and encouraged in projects, where the work is explained and defended; it is excluded from the two tests, which certify unaided capability.</t>
         </is>
       </c>
       <c r="H11" s="54" t="inlineStr">
         <is>
-          <t>The test is the practical. Duration 2h00 practical + 0h25 written. Three parallel dataset variants are issued in a checkerboard seating pattern to remove any benefit from collusion.</t>
+          <t>The test is a coding practical in Colab, three hours from the start including setup, checking and submission. Three parallel dataset variants are issued by the entry page, and the deterministic grader re-runs the submitted code on other data.</t>
         </is>
       </c>
       <c r="I11" s="54" t="inlineStr">
@@ -5571,26 +5589,24 @@
       </c>
       <c r="M11" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 1 = 15% of the Semester 1 mark. Individual. Rubric: profiling 15, cleaning decisions and justification 20, visualisation 20, findings correctness 20, engineering interpretation 15, notebook clarity and reproducibility 10.</t>
+          <t>PRACTICAL TEST 1 = 15% of the Semester 1 mark. Individual. Rubric: reading and inspecting 20, chart before cleaning 10, cleaning 20, chart after cleaning 10, statistics 15, grouping 10, one function 5, conditions and a loop 10.</t>
         </is>
       </c>
       <c r="N11" s="54" t="inlineStr">
         <is>
-          <t>• CAPACITY PLAN: confirm machine and seat availability against cohort size now. Cohort A (~100) will very likely require two sittings with different dataset variants, or a BYOD-plus-lab hybrid. Escalate to the Faculty in Week 1, not Week 6.
-• Author three parallel dataset variants of matched difficulty, plus a model answer and a mark scheme for each.
-• Build the offline bundle: datasets, offline pandas/seaborn documentation, task sheet. Test it on a machine with the network cable physically unplugged.
-• Prepare the invigilation plan, seating chart, and a submission collection method that works without a network (USB collection or a local drop folder).
-• Write a structural auto-check script (does the notebook run top to bottom? are the required sections present?) to make ~100 scripts markable in reasonable time.
-• Agree the moderation plan and the late/absent policy with the Faculty in advance.</t>
+          <t>• Author three parallel dataset variants of matched difficulty, and the hidden data the grader uses.
+• Test the entry page, private notebook, countdown, Submit test button and form link with one account for each variant.
+• Confirm that every student has a Google account that works with Colab and the submission form.
+• The deterministic grader marks all eight tasks, so no structural auto-check script is needed.
+• Agree the moderation plan and the late and absent policy with the Faculty in advance.</t>
         </is>
       </c>
       <c r="O11" s="54" t="inlineStr">
         <is>
-          <t>• Invigilated lab, offline. Confirmed machine count. Spare machines and a power contingency.
-• USB drives or a local drop folder for collection.
-• Printed task sheets (one per variant) and typed notebook response cells for Part B.
-• Second invigilator for any sitting above 40 students.
-• Published rubric (issued Week 6).</t>
+          <t>• A Colab-capable laptop and a stable connection for every student.
+• An entry link or QR code for each variant.
+• Published rubric (issued Week 6).
+• A short understanding check for a sample of students after the test.</t>
         </is>
       </c>
     </row>
@@ -6223,25 +6239,24 @@
       </c>
       <c r="C18" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, offline)</t>
+          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="D18" s="54" t="inlineStr">
         <is>
-          <t>• Frame an unfamiliar engineering problem as a machine learning task, unaided.
-• Prepare data and control leakage within a pipeline.
-• Build and compare at least two models under a single valid protocol.
-• Evaluate with a justified metric and report the result in engineering terms.
-• State the model's limitations and the conditions under which it should not be used.
-• Explain their own reasoning in writing without any tool.</t>
+          <t>• Split data by whole equipment groups and fit models on training rows only.
+• Compare a baseline, a straight line, a tree, a ridge curve and nearest neighbours on the same validation rows.
+• Count classification outcomes and work out a cost, and run cross-validation by group.
+• Test whether an extra input helps, and choose a model inside stated limits.
+• Explain the choices: sealed test rows, training-only fill values, scaling and the ridge penalty.</t>
         </is>
       </c>
       <c r="E18" s="54" t="inlineStr">
         <is>
-          <t>• 0:00-0:15  Seating, machine allocation, variant distribution, rules read aloud, offline mode confirmed.
-• 0:15-2:15  TEST, PART A (practical, 2 hours). Individual, unfamiliar dataset from the cohort's domain. Tasks: state the ML task and name the target; prepare the data with justified decisions; build at least two models inside a leak-proof pipeline; evaluate with a justified metric and validate properly; report the result in physical or operational units; state three limitations.
-• 2:15-2:40  TEST, PART B (written reasoning, 25 minutes, typed offline responses only; no code execution). Why this metric. Where could this pipeline leak. What would change your recommendation. Would you deploy this, and what would you require first.
-• 2:40-3:00  Collection, structural check, dismissal. Week 15 demo running order confirmed.</t>
+          <t>• 0:00-0:15  Entry page, notebook and CSV downloaded, rules read aloud, identity cell checked.
+• 0:15-2:15  CODING (120 minutes). Individual, in Colab. Eight functions covering Weeks 8 to 13, from group_split to ridge_and_knn. The notebook states the columns, return formats and marks.
+• 2:15-2:40  INTERPRETATION AND CHECKING (25 minutes). Six scenario choices recorded in DECISIONS, then Restart and Run all.
+• 2:40-3:00  FINAL SAVE AND SUBMISSION (20 minutes). Submit test button, generated form link, confirmation. Week 15 demo running order confirmed.</t>
         </is>
       </c>
       <c r="F18" s="54" t="inlineStr">
@@ -6251,14 +6266,14 @@
       </c>
       <c r="G18" s="54" t="inlineStr">
         <is>
-          <t>• Permitted: Python, VS Code or Jupyter, pandas, NumPy, matplotlib, seaborn, scikit-learn, and the offline documentation bundle.
-• Prohibited: internet, AI assistants, messaging. The room runs offline.
-• The offline bundle must include the scikit-learn API documentation - the test examines judgement, not memory of parameter names.</t>
+          <t>• Permitted: Colab, the submission form and any other resource the invigilator announces.
+• Prohibited: AI assistants, messaging and copied answers.
+• The notebook explains the columns and return formats, so the test examines judgement rather than memory of parameter names.</t>
         </is>
       </c>
       <c r="H18" s="54" t="inlineStr">
         <is>
-          <t>The test is the practical. Duration 2h00 practical + 0h25 written. Three parallel dataset variants in a checkerboard seating pattern.</t>
+          <t>The test is a coding practical in Colab, three hours from the start including setup, checking and submission. Three parallel dataset variants are issued by the entry page, and the deterministic grader re-runs the submitted code on other data.</t>
         </is>
       </c>
       <c r="I18" s="54" t="inlineStr">
@@ -6283,24 +6298,22 @@
       </c>
       <c r="M18" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 2 = 20% of the Semester 1 mark. Individual. Rubric: task framing 10, data preparation and leakage control 20, modelling protocol 20, evaluation and metric justification 20, engineering interpretation and limits 20, code clarity 10.</t>
+          <t>PRACTICAL TEST 2 = 20% of the Semester 1 mark. Individual. Rubric: group split 10, baseline, linear and tree predictions 15, MAE and RMSE 5, classification and cost 10, group cross-validation 10, feature ablation 10, model selection 10, ridge and nearest neighbours 15, six interpretation choices 15.</t>
         </is>
       </c>
       <c r="N18" s="54" t="inlineStr">
         <is>
-          <t>• Author three parallel dataset variants of matched difficulty, each with a model answer and a mark scheme.
-• Build and test the offline bundle, including scikit-learn documentation, on a machine with the network physically disconnected.
-• Confirm the capacity plan. Cohort A will very likely need two sittings; this must be timetabled with the Faculty by Week 7 at the latest.
-• Write the structural auto-check script (runs top to bottom, required sections present, no internet calls) to make large-cohort marking feasible.
-• Agree the moderation sample and the double-marking plan with the Faculty.
+          <t>• Author three parallel dataset variants of matched difficulty, each with a reference solution. The grader re-runs submitted code on unseen data.
+• Test the entry page, notebook download, Submit test button and form link with one account for each variant.
+• Confirm sittings, invigilators and Colab capacity with the Faculty. Cohort A is about 100 students.
+• Agree the moderation sample with the Faculty.
 • Prepare the Week 15 demo running order, two typed defence prompts and the digital submission check.</t>
         </is>
       </c>
       <c r="O18" s="54" t="inlineStr">
         <is>
-          <t>• Invigilated offline lab; confirmed machine count; spare machines; power contingency.
-• USB or local drop folder collection.
-• Printed task sheets per variant; Part B answers typed into the notebook.
+          <t>• A room with stable wifi and a Colab-capable laptop for every student; confirmed seat count; power contingency.
+• Entry links or QR codes for each variant.
 • Second invigilator for any sitting above 40 students.
 • Rubric published in Week 11.</t>
         </is>
@@ -6465,6 +6478,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="43.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -7438,25 +7452,23 @@
       </c>
       <c r="H11" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 1 - Data Investigation (individual, offline)</t>
+          <t>PRACTICAL TEST 1 - Data Investigation (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="I11" s="54" t="inlineStr">
         <is>
-          <t>• Independently investigate an unfamiliar engineering dataset under time pressure.
-• Profile, clean and justify, without a prescribed method.
-• Answer stated questions with evidence and correct units.
-• Produce charts that answer questions.
-• Draw an engineering conclusion and state what further data would be needed.
-• Explain their own reasoning in typed offline responses, without executing code or using AI.</t>
+          <t>• Read, inspect and clean an unfamiliar engineering dataset without a prescribed method, and check the result with charts.
+• Calculate summary statistics and group means with pandas and report them accurately.
+• Write a function that works on any table, and a loop with conditions.
+• Explain their own submitted code when asked, without AI or another person's help.</t>
         </is>
       </c>
       <c r="J11" s="54" t="inlineStr">
         <is>
-          <t>• 0:00-0:15  Seating, machine allocation, dataset variant distribution, rules read aloud, offline mode confirmed.
-• 0:15-2:15  TEST, PART A (practical, 2 hours). Individual. An unfamiliar dataset from the cohort's domain plus a task sheet: load and profile; identify and handle defects with a written justification for each; answer three stated engineering questions with evidence; produce three charts, each captioned with the question it answers; list five findings; make one engineering recommendation.
-• 2:15-2:40  TEST, PART B (written reasoning, 25 minutes, typed offline responses only; no code execution). Four short questions on their own submission: why that cleaning decision, what the chart does not show, what would change the conclusion, and what data is missing.
-• 2:40-3:00  Collection, checksum of submissions, immediate structural check, dismissal.</t>
+          <t>• 0:00-0:10  Entry link, private notebook and CSV, rules read aloud, identity cell checked.
+• 0:10-2:25  CODING (135 minutes). Individual, in Colab. Eight coded tasks: read and inspect the file, a chart before cleaning, cleaning, a chart after cleaning, statistics, grouping, one function, and a loop with conditions.
+• 2:25-2:40  CHECKING (15 minutes). Restart the session and Run all.
+• 2:40-3:00  FINAL SAVE AND SUBMISSION (20 minutes). Submit test button, generated form link, confirmation.</t>
         </is>
       </c>
       <c r="K11" s="54" t="inlineStr">
@@ -7467,14 +7479,14 @@
       </c>
       <c r="L11" s="54" t="inlineStr">
         <is>
-          <t>• Permitted: Python, VS Code or Jupyter, pandas, NumPy, matplotlib, seaborn, and an OFFLINE documentation bundle.
-• Prohibited: internet access, AI assistants, messaging and shared drives. Use the invigilated offline lab and approved-materials checks; offline access alone does not prevent a local AI assistant.
+          <t>• Permitted: Colab, pandas, matplotlib, ordinary Python, and your lecture slides, revision guide, cheatsheet and personal course notes.
+• Prohibited: AI tools, help from another person and copied work. Colab cannot block an AI assistant, so the rule rests on the declaration, hidden-data grading and an understanding check in which a student may be asked to explain or change their own code.
 • Rationale published to students in Week 6: AI is permitted and encouraged in projects, where the work is explained and defended; it is excluded from the two tests, which certify unaided capability.</t>
         </is>
       </c>
       <c r="M11" s="54" t="inlineStr">
         <is>
-          <t>The test is the practical. Duration 2h00 practical + 0h25 written. Three parallel dataset variants are issued in a checkerboard seating pattern to remove any benefit from collusion.</t>
+          <t>The test is a coding practical in Colab, three hours from the start including setup, checking and submission. Three parallel dataset variants are issued by the entry page, and the deterministic grader re-runs the submitted code on other data.</t>
         </is>
       </c>
       <c r="N11" s="54" t="inlineStr">
@@ -7504,31 +7516,29 @@
       </c>
       <c r="S11" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 1 = 15% of the Semester 1 mark. Individual. Rubric: profiling 15, cleaning decisions and justification 20, visualisation 20, findings correctness 20, engineering interpretation 15, notebook clarity and reproducibility 10.</t>
+          <t>PRACTICAL TEST 1 = 15% of the Semester 1 mark. Individual. Rubric: reading and inspecting 20, chart before cleaning 10, cleaning 20, chart after cleaning 10, statistics 15, grouping 10, one function 5, conditions and a loop 10.</t>
         </is>
       </c>
       <c r="T11" s="54" t="inlineStr">
         <is>
-          <t>• CAPACITY PLAN: confirm machine and seat availability against cohort size now. Cohort A (~100) will very likely require two sittings with different dataset variants, or a BYOD-plus-lab hybrid. Escalate to the Faculty in Week 1, not Week 6.
-• Author three parallel dataset variants of matched difficulty, plus a model answer and a mark scheme for each.
-• Build the offline bundle: datasets, offline pandas/seaborn documentation, task sheet. Test it on a machine with the network cable physically unplugged.
-• Prepare the invigilation plan, seating chart, and a submission collection method that works without a network (USB collection or a local drop folder).
-• Write a structural auto-check script (does the notebook run top to bottom? are the required sections present?) to make ~100 scripts markable in reasonable time.
-• Agree the moderation plan and the late/absent policy with the Faculty in advance.</t>
+          <t>• Author three parallel dataset variants of matched difficulty, and the hidden data the grader uses.
+• Test the entry page, private notebook, countdown, Submit test button and form link with one account for each variant.
+• Confirm that every student has a Google account that works with Colab and the submission form.
+• The deterministic grader marks all eight tasks, so no structural auto-check script is needed.
+• Agree the moderation plan and the late and absent policy with the Faculty in advance.</t>
         </is>
       </c>
       <c r="U11" s="54" t="inlineStr">
         <is>
-          <t>• Invigilated lab, offline. Confirmed machine count. Spare machines and a power contingency.
-• USB drives or a local drop folder for collection.
-• Printed task sheets (one per variant) and typed notebook response cells for Part B.
-• Second invigilator for any sitting above 40 students.
-• Published rubric (issued Week 6).</t>
+          <t>• A Colab-capable laptop and a stable connection for every student.
+• An entry link or QR code for each variant.
+• Published rubric (issued Week 6).
+• A short understanding check for a sample of students after the test.</t>
         </is>
       </c>
       <c r="V11" s="54" t="inlineStr">
         <is>
-          <t>DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, offline bundle.</t>
+          <t>DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, issued notebook bundle.</t>
         </is>
       </c>
     </row>
@@ -8406,25 +8416,24 @@
       </c>
       <c r="H18" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, offline)</t>
+          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="I18" s="54" t="inlineStr">
         <is>
-          <t>• Frame an unfamiliar engineering problem as a machine learning task, unaided.
-• Prepare data and control leakage within a pipeline.
-• Build and compare at least two models under a single valid protocol.
-• Evaluate with a justified metric and report the result in engineering terms.
-• State the model's limitations and the conditions under which it should not be used.
-• Explain their own reasoning in writing without any tool.</t>
+          <t>• Split data by whole equipment groups and fit models on training rows only.
+• Compare a baseline, a straight line, a tree, a ridge curve and nearest neighbours on the same validation rows.
+• Count classification outcomes and work out a cost, and run cross-validation by group.
+• Test whether an extra input helps, and choose a model inside stated limits.
+• Explain the choices: sealed test rows, training-only fill values, scaling and the ridge penalty.</t>
         </is>
       </c>
       <c r="J18" s="54" t="inlineStr">
         <is>
-          <t>• 0:00-0:15  Seating, machine allocation, variant distribution, rules read aloud, offline mode confirmed.
-• 0:15-2:15  TEST, PART A (practical, 2 hours). Individual, unfamiliar dataset from the cohort's domain. Tasks: state the ML task and name the target; prepare the data with justified decisions; build at least two models inside a leak-proof pipeline; evaluate with a justified metric and validate properly; report the result in physical or operational units; state three limitations.
-• 2:15-2:40  TEST, PART B (written reasoning, 25 minutes, typed offline responses only; no code execution). Why this metric. Where could this pipeline leak. What would change your recommendation. Would you deploy this, and what would you require first.
-• 2:40-3:00  Collection, structural check, dismissal. Week 15 demo running order confirmed.</t>
+          <t>• 0:00-0:15  Entry page, notebook and CSV downloaded, rules read aloud, identity cell checked.
+• 0:15-2:15  CODING (120 minutes). Individual, in Colab. Eight functions covering Weeks 8 to 13, from group_split to ridge_and_knn. The notebook states the columns, return formats and marks.
+• 2:15-2:40  INTERPRETATION AND CHECKING (25 minutes). Six scenario choices recorded in DECISIONS, then Restart and Run all.
+• 2:40-3:00  FINAL SAVE AND SUBMISSION (20 minutes). Submit test button, generated form link, confirmation. Week 15 demo running order confirmed.</t>
         </is>
       </c>
       <c r="K18" s="54" t="inlineStr">
@@ -8434,14 +8443,14 @@
       </c>
       <c r="L18" s="54" t="inlineStr">
         <is>
-          <t>• Permitted: Python, VS Code or Jupyter, pandas, NumPy, matplotlib, seaborn, scikit-learn, and the offline documentation bundle.
-• Prohibited: internet, AI assistants, messaging. The room runs offline.
-• The offline bundle must include the scikit-learn API documentation - the test examines judgement, not memory of parameter names.</t>
+          <t>• Permitted: Colab, the submission form and any other resource the invigilator announces.
+• Prohibited: AI assistants, messaging and copied answers.
+• The notebook explains the columns and return formats, so the test examines judgement rather than memory of parameter names.</t>
         </is>
       </c>
       <c r="M18" s="54" t="inlineStr">
         <is>
-          <t>The test is the practical. Duration 2h00 practical + 0h25 written. Three parallel dataset variants in a checkerboard seating pattern.</t>
+          <t>The test is a coding practical in Colab, three hours from the start including setup, checking and submission. Three parallel dataset variants are issued by the entry page, and the deterministic grader re-runs the submitted code on other data.</t>
         </is>
       </c>
       <c r="N18" s="54" t="inlineStr">
@@ -8471,24 +8480,22 @@
       </c>
       <c r="S18" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 2 = 20% of the Semester 1 mark. Individual. Rubric: task framing 10, data preparation and leakage control 20, modelling protocol 20, evaluation and metric justification 20, engineering interpretation and limits 20, code clarity 10.</t>
+          <t>PRACTICAL TEST 2 = 20% of the Semester 1 mark. Individual. Rubric: group split 10, baseline, linear and tree predictions 15, MAE and RMSE 5, classification and cost 10, group cross-validation 10, feature ablation 10, model selection 10, ridge and nearest neighbours 15, six interpretation choices 15.</t>
         </is>
       </c>
       <c r="T18" s="54" t="inlineStr">
         <is>
-          <t>• Author three parallel dataset variants of matched difficulty, each with a model answer and a mark scheme.
-• Build and test the offline bundle, including scikit-learn documentation, on a machine with the network physically disconnected.
-• Confirm the capacity plan. Cohort A will very likely need two sittings; this must be timetabled with the Faculty by Week 7 at the latest.
-• Write the structural auto-check script (runs top to bottom, required sections present, no internet calls) to make large-cohort marking feasible.
-• Agree the moderation sample and the double-marking plan with the Faculty.
+          <t>• Author three parallel dataset variants of matched difficulty, each with a reference solution. The grader re-runs submitted code on unseen data.
+• Test the entry page, notebook download, Submit test button and form link with one account for each variant.
+• Confirm sittings, invigilators and Colab capacity with the Faculty. Cohort A is about 100 students.
+• Agree the moderation sample with the Faculty.
 • Prepare the Week 15 demo running order, two typed defence prompts and the digital submission check.</t>
         </is>
       </c>
       <c r="U18" s="54" t="inlineStr">
         <is>
-          <t>• Invigilated offline lab; confirmed machine count; spare machines; power contingency.
-• USB or local drop folder collection.
-• Printed task sheets per variant; Part B answers typed into the notebook.
+          <t>• A room with stable wifi and a Colab-capable laptop for every student; confirmed seat count; power contingency.
+• Entry links or QR codes for each variant.
 • Second invigilator for any sitting above 40 students.
 • Rubric published in Week 11.</t>
         </is>
@@ -8694,6 +8701,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="43.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -9668,25 +9676,23 @@
       </c>
       <c r="H11" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 1 - Data Investigation (individual, offline)</t>
+          <t>PRACTICAL TEST 1 - Data Investigation (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="I11" s="54" t="inlineStr">
         <is>
-          <t>• Independently investigate an unfamiliar engineering dataset under time pressure.
-• Profile, clean and justify, without a prescribed method.
-• Answer stated questions with evidence and correct units.
-• Produce charts that answer questions.
-• Draw an engineering conclusion and state what further data would be needed.
-• Explain their own reasoning in typed offline responses, without executing code or using AI.</t>
+          <t>• Read, inspect and clean an unfamiliar engineering dataset without a prescribed method, and check the result with charts.
+• Calculate summary statistics and group means with pandas and report them accurately.
+• Write a function that works on any table, and a loop with conditions.
+• Explain their own submitted code when asked, without AI or another person's help.</t>
         </is>
       </c>
       <c r="J11" s="54" t="inlineStr">
         <is>
-          <t>• 0:00-0:15  Seating, machine allocation, dataset variant distribution, rules read aloud, offline mode confirmed.
-• 0:15-2:15  TEST, PART A (practical, 2 hours). Individual. An unfamiliar dataset from the cohort's domain plus a task sheet: load and profile; identify and handle defects with a written justification for each; answer three stated engineering questions with evidence; produce three charts, each captioned with the question it answers; list five findings; make one engineering recommendation.
-• 2:15-2:40  TEST, PART B (written reasoning, 25 minutes, typed offline responses only; no code execution). Four short questions on their own submission: why that cleaning decision, what the chart does not show, what would change the conclusion, and what data is missing.
-• 2:40-3:00  Collection, checksum of submissions, immediate structural check, dismissal.</t>
+          <t>• 0:00-0:10  Entry link, private notebook and CSV, rules read aloud, identity cell checked.
+• 0:10-2:25  CODING (135 minutes). Individual, in Colab. Eight coded tasks: read and inspect the file, a chart before cleaning, cleaning, a chart after cleaning, statistics, grouping, one function, and a loop with conditions.
+• 2:25-2:40  CHECKING (15 minutes). Restart the session and Run all.
+• 2:40-3:00  FINAL SAVE AND SUBMISSION (20 minutes). Submit test button, generated form link, confirmation.</t>
         </is>
       </c>
       <c r="K11" s="54" t="inlineStr">
@@ -9697,14 +9703,14 @@
       </c>
       <c r="L11" s="54" t="inlineStr">
         <is>
-          <t>• Permitted: Python, VS Code or Jupyter, pandas, NumPy, matplotlib, seaborn, and an OFFLINE documentation bundle.
-• Prohibited: internet access, AI assistants, messaging and shared drives. Use the invigilated offline lab and approved-materials checks; offline access alone does not prevent a local AI assistant.
+          <t>• Permitted: Colab, pandas, matplotlib, ordinary Python, and your lecture slides, revision guide, cheatsheet and personal course notes.
+• Prohibited: AI tools, help from another person and copied work. Colab cannot block an AI assistant, so the rule rests on the declaration, hidden-data grading and an understanding check in which a student may be asked to explain or change their own code.
 • Rationale published to students in Week 6: AI is permitted and encouraged in projects, where the work is explained and defended; it is excluded from the two tests, which certify unaided capability.</t>
         </is>
       </c>
       <c r="M11" s="54" t="inlineStr">
         <is>
-          <t>The test is the practical. Duration 2h00 practical + 0h25 written. Three parallel dataset variants are issued in a checkerboard seating pattern to remove any benefit from collusion.</t>
+          <t>The test is a coding practical in Colab, three hours from the start including setup, checking and submission. Three parallel dataset variants are issued by the entry page, and the deterministic grader re-runs the submitted code on other data.</t>
         </is>
       </c>
       <c r="N11" s="54" t="inlineStr">
@@ -9734,31 +9740,29 @@
       </c>
       <c r="S11" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 1 = 15% of the Semester 1 mark. Individual. Rubric: profiling 15, cleaning decisions and justification 20, visualisation 20, findings correctness 20, engineering interpretation 15, notebook clarity and reproducibility 10.</t>
+          <t>PRACTICAL TEST 1 = 15% of the Semester 1 mark. Individual. Rubric: reading and inspecting 20, chart before cleaning 10, cleaning 20, chart after cleaning 10, statistics 15, grouping 10, one function 5, conditions and a loop 10.</t>
         </is>
       </c>
       <c r="T11" s="54" t="inlineStr">
         <is>
-          <t>• CAPACITY PLAN: confirm machine and seat availability against cohort size now. Cohort A (~100) will very likely require two sittings with different dataset variants, or a BYOD-plus-lab hybrid. Escalate to the Faculty in Week 1, not Week 6.
-• Author three parallel dataset variants of matched difficulty, plus a model answer and a mark scheme for each.
-• Build the offline bundle: datasets, offline pandas/seaborn documentation, task sheet. Test it on a machine with the network cable physically unplugged.
-• Prepare the invigilation plan, seating chart, and a submission collection method that works without a network (USB collection or a local drop folder).
-• Write a structural auto-check script (does the notebook run top to bottom? are the required sections present?) to make ~100 scripts markable in reasonable time.
-• Agree the moderation plan and the late/absent policy with the Faculty in advance.</t>
+          <t>• Author three parallel dataset variants of matched difficulty, and the hidden data the grader uses.
+• Test the entry page, private notebook, countdown, Submit test button and form link with one account for each variant.
+• Confirm that every student has a Google account that works with Colab and the submission form.
+• The deterministic grader marks all eight tasks, so no structural auto-check script is needed.
+• Agree the moderation plan and the late and absent policy with the Faculty in advance.</t>
         </is>
       </c>
       <c r="U11" s="54" t="inlineStr">
         <is>
-          <t>• Invigilated lab, offline. Confirmed machine count. Spare machines and a power contingency.
-• USB drives or a local drop folder for collection.
-• Printed task sheets (one per variant) and typed notebook response cells for Part B.
-• Second invigilator for any sitting above 40 students.
-• Published rubric (issued Week 6).</t>
+          <t>• A Colab-capable laptop and a stable connection for every student.
+• An entry link or QR code for each variant.
+• Published rubric (issued Week 6).
+• A short understanding check for a sample of students after the test.</t>
         </is>
       </c>
       <c r="V11" s="54" t="inlineStr">
         <is>
-          <t>DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, offline bundle.</t>
+          <t>DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, issued notebook bundle.</t>
         </is>
       </c>
     </row>
@@ -10636,25 +10640,24 @@
       </c>
       <c r="H18" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, offline)</t>
+          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="I18" s="54" t="inlineStr">
         <is>
-          <t>• Frame an unfamiliar engineering problem as a machine learning task, unaided.
-• Prepare data and control leakage within a pipeline.
-• Build and compare at least two models under a single valid protocol.
-• Evaluate with a justified metric and report the result in engineering terms.
-• State the model's limitations and the conditions under which it should not be used.
-• Explain their own reasoning in writing without any tool.</t>
+          <t>• Split data by whole equipment groups and fit models on training rows only.
+• Compare a baseline, a straight line, a tree, a ridge curve and nearest neighbours on the same validation rows.
+• Count classification outcomes and work out a cost, and run cross-validation by group.
+• Test whether an extra input helps, and choose a model inside stated limits.
+• Explain the choices: sealed test rows, training-only fill values, scaling and the ridge penalty.</t>
         </is>
       </c>
       <c r="J18" s="54" t="inlineStr">
         <is>
-          <t>• 0:00-0:15  Seating, machine allocation, variant distribution, rules read aloud, offline mode confirmed.
-• 0:15-2:15  TEST, PART A (practical, 2 hours). Individual, unfamiliar dataset from the cohort's domain. Tasks: state the ML task and name the target; prepare the data with justified decisions; build at least two models inside a leak-proof pipeline; evaluate with a justified metric and validate properly; report the result in physical or operational units; state three limitations.
-• 2:15-2:40  TEST, PART B (written reasoning, 25 minutes, typed offline responses only; no code execution). Why this metric. Where could this pipeline leak. What would change your recommendation. Would you deploy this, and what would you require first.
-• 2:40-3:00  Collection, structural check, dismissal. Week 15 demo running order confirmed.</t>
+          <t>• 0:00-0:15  Entry page, notebook and CSV downloaded, rules read aloud, identity cell checked.
+• 0:15-2:15  CODING (120 minutes). Individual, in Colab. Eight functions covering Weeks 8 to 13, from group_split to ridge_and_knn. The notebook states the columns, return formats and marks.
+• 2:15-2:40  INTERPRETATION AND CHECKING (25 minutes). Six scenario choices recorded in DECISIONS, then Restart and Run all.
+• 2:40-3:00  FINAL SAVE AND SUBMISSION (20 minutes). Submit test button, generated form link, confirmation. Week 15 demo running order confirmed.</t>
         </is>
       </c>
       <c r="K18" s="54" t="inlineStr">
@@ -10664,14 +10667,14 @@
       </c>
       <c r="L18" s="54" t="inlineStr">
         <is>
-          <t>• Permitted: Python, VS Code or Jupyter, pandas, NumPy, matplotlib, seaborn, scikit-learn, and the offline documentation bundle.
-• Prohibited: internet, AI assistants, messaging. The room runs offline.
-• The offline bundle must include the scikit-learn API documentation - the test examines judgement, not memory of parameter names.</t>
+          <t>• Permitted: Colab, the submission form and any other resource the invigilator announces.
+• Prohibited: AI assistants, messaging and copied answers.
+• The notebook explains the columns and return formats, so the test examines judgement rather than memory of parameter names.</t>
         </is>
       </c>
       <c r="M18" s="54" t="inlineStr">
         <is>
-          <t>The test is the practical. Duration 2h00 practical + 0h25 written. Three parallel dataset variants in a checkerboard seating pattern.</t>
+          <t>The test is a coding practical in Colab, three hours from the start including setup, checking and submission. Three parallel dataset variants are issued by the entry page, and the deterministic grader re-runs the submitted code on other data.</t>
         </is>
       </c>
       <c r="N18" s="54" t="inlineStr">
@@ -10701,24 +10704,22 @@
       </c>
       <c r="S18" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 2 = 20% of the Semester 1 mark. Individual. Rubric: task framing 10, data preparation and leakage control 20, modelling protocol 20, evaluation and metric justification 20, engineering interpretation and limits 20, code clarity 10.</t>
+          <t>PRACTICAL TEST 2 = 20% of the Semester 1 mark. Individual. Rubric: group split 10, baseline, linear and tree predictions 15, MAE and RMSE 5, classification and cost 10, group cross-validation 10, feature ablation 10, model selection 10, ridge and nearest neighbours 15, six interpretation choices 15.</t>
         </is>
       </c>
       <c r="T18" s="54" t="inlineStr">
         <is>
-          <t>• Author three parallel dataset variants of matched difficulty, each with a model answer and a mark scheme.
-• Build and test the offline bundle, including scikit-learn documentation, on a machine with the network physically disconnected.
-• Confirm the capacity plan. Cohort A will very likely need two sittings; this must be timetabled with the Faculty by Week 7 at the latest.
-• Write the structural auto-check script (runs top to bottom, required sections present, no internet calls) to make large-cohort marking feasible.
-• Agree the moderation sample and the double-marking plan with the Faculty.
+          <t>• Author three parallel dataset variants of matched difficulty, each with a reference solution. The grader re-runs submitted code on unseen data.
+• Test the entry page, notebook download, Submit test button and form link with one account for each variant.
+• Confirm sittings, invigilators and Colab capacity with the Faculty. Cohort A is about 100 students.
+• Agree the moderation sample with the Faculty.
 • Prepare the Week 15 demo running order, two typed defence prompts and the digital submission check.</t>
         </is>
       </c>
       <c r="U18" s="54" t="inlineStr">
         <is>
-          <t>• Invigilated offline lab; confirmed machine count; spare machines; power contingency.
-• USB or local drop folder collection.
-• Printed task sheets per variant; Part B answers typed into the notebook.
+          <t>• A room with stable wifi and a Colab-capable laptop for every student; confirmed seat count; power contingency.
+• Entry links or QR codes for each variant.
 • Second invigilator for any sitting above 40 students.
 • Rubric published in Week 11.</t>
         </is>
@@ -10924,6 +10925,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="43.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -11897,25 +11899,23 @@
       </c>
       <c r="H11" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 1 - Data Investigation (individual, offline)</t>
+          <t>PRACTICAL TEST 1 - Data Investigation (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="I11" s="54" t="inlineStr">
         <is>
-          <t>• Independently investigate an unfamiliar engineering dataset under time pressure.
-• Profile, clean and justify, without a prescribed method.
-• Answer stated questions with evidence and correct units.
-• Produce charts that answer questions.
-• Draw an engineering conclusion and state what further data would be needed.
-• Explain their own reasoning in typed offline responses, without executing code or using AI.</t>
+          <t>• Read, inspect and clean an unfamiliar engineering dataset without a prescribed method, and check the result with charts.
+• Calculate summary statistics and group means with pandas and report them accurately.
+• Write a function that works on any table, and a loop with conditions.
+• Explain their own submitted code when asked, without AI or another person's help.</t>
         </is>
       </c>
       <c r="J11" s="54" t="inlineStr">
         <is>
-          <t>• 0:00-0:15  Seating, machine allocation, dataset variant distribution, rules read aloud, offline mode confirmed.
-• 0:15-2:15  TEST, PART A (practical, 2 hours). Individual. An unfamiliar dataset from the cohort's domain plus a task sheet: load and profile; identify and handle defects with a written justification for each; answer three stated engineering questions with evidence; produce three charts, each captioned with the question it answers; list five findings; make one engineering recommendation.
-• 2:15-2:40  TEST, PART B (written reasoning, 25 minutes, typed offline responses only; no code execution). Four short questions on their own submission: why that cleaning decision, what the chart does not show, what would change the conclusion, and what data is missing.
-• 2:40-3:00  Collection, checksum of submissions, immediate structural check, dismissal.</t>
+          <t>• 0:00-0:10  Entry link, private notebook and CSV, rules read aloud, identity cell checked.
+• 0:10-2:25  CODING (135 minutes). Individual, in Colab. Eight coded tasks: read and inspect the file, a chart before cleaning, cleaning, a chart after cleaning, statistics, grouping, one function, and a loop with conditions.
+• 2:25-2:40  CHECKING (15 minutes). Restart the session and Run all.
+• 2:40-3:00  FINAL SAVE AND SUBMISSION (20 minutes). Submit test button, generated form link, confirmation.</t>
         </is>
       </c>
       <c r="K11" s="54" t="inlineStr">
@@ -11926,14 +11926,14 @@
       </c>
       <c r="L11" s="54" t="inlineStr">
         <is>
-          <t>• Permitted: Python, VS Code or Jupyter, pandas, NumPy, matplotlib, seaborn, and an OFFLINE documentation bundle.
-• Prohibited: internet access, AI assistants, messaging and shared drives. Use the invigilated offline lab and approved-materials checks; offline access alone does not prevent a local AI assistant.
+          <t>• Permitted: Colab, pandas, matplotlib, ordinary Python, and your lecture slides, revision guide, cheatsheet and personal course notes.
+• Prohibited: AI tools, help from another person and copied work. Colab cannot block an AI assistant, so the rule rests on the declaration, hidden-data grading and an understanding check in which a student may be asked to explain or change their own code.
 • Rationale published to students in Week 6: AI is permitted and encouraged in projects, where the work is explained and defended; it is excluded from the two tests, which certify unaided capability.</t>
         </is>
       </c>
       <c r="M11" s="54" t="inlineStr">
         <is>
-          <t>The test is the practical. Duration 2h00 practical + 0h25 written. Three parallel dataset variants are issued in a checkerboard seating pattern to remove any benefit from collusion.</t>
+          <t>The test is a coding practical in Colab, three hours from the start including setup, checking and submission. Three parallel dataset variants are issued by the entry page, and the deterministic grader re-runs the submitted code on other data.</t>
         </is>
       </c>
       <c r="N11" s="54" t="inlineStr">
@@ -11963,31 +11963,29 @@
       </c>
       <c r="S11" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 1 = 15% of the Semester 1 mark. Individual. Rubric: profiling 15, cleaning decisions and justification 20, visualisation 20, findings correctness 20, engineering interpretation 15, notebook clarity and reproducibility 10.</t>
+          <t>PRACTICAL TEST 1 = 15% of the Semester 1 mark. Individual. Rubric: reading and inspecting 20, chart before cleaning 10, cleaning 20, chart after cleaning 10, statistics 15, grouping 10, one function 5, conditions and a loop 10.</t>
         </is>
       </c>
       <c r="T11" s="54" t="inlineStr">
         <is>
-          <t>• CAPACITY PLAN: confirm machine and seat availability against cohort size now. Cohort A (~100) will very likely require two sittings with different dataset variants, or a BYOD-plus-lab hybrid. Escalate to the Faculty in Week 1, not Week 6.
-• Author three parallel dataset variants of matched difficulty, plus a model answer and a mark scheme for each.
-• Build the offline bundle: datasets, offline pandas/seaborn documentation, task sheet. Test it on a machine with the network cable physically unplugged.
-• Prepare the invigilation plan, seating chart, and a submission collection method that works without a network (USB collection or a local drop folder).
-• Write a structural auto-check script (does the notebook run top to bottom? are the required sections present?) to make ~100 scripts markable in reasonable time.
-• Agree the moderation plan and the late/absent policy with the Faculty in advance.</t>
+          <t>• Author three parallel dataset variants of matched difficulty, and the hidden data the grader uses.
+• Test the entry page, private notebook, countdown, Submit test button and form link with one account for each variant.
+• Confirm that every student has a Google account that works with Colab and the submission form.
+• The deterministic grader marks all eight tasks, so no structural auto-check script is needed.
+• Agree the moderation plan and the late and absent policy with the Faculty in advance.</t>
         </is>
       </c>
       <c r="U11" s="54" t="inlineStr">
         <is>
-          <t>• Invigilated lab, offline. Confirmed machine count. Spare machines and a power contingency.
-• USB drives or a local drop folder for collection.
-• Printed task sheets (one per variant) and typed notebook response cells for Part B.
-• Second invigilator for any sitting above 40 students.
-• Published rubric (issued Week 6).</t>
+          <t>• A Colab-capable laptop and a stable connection for every student.
+• An entry link or QR code for each variant.
+• Published rubric (issued Week 6).
+• A short understanding check for a sample of students after the test.</t>
         </is>
       </c>
       <c r="V11" s="54" t="inlineStr">
         <is>
-          <t>DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, offline bundle.</t>
+          <t>DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, issued notebook bundle.</t>
         </is>
       </c>
     </row>
@@ -12865,25 +12863,24 @@
       </c>
       <c r="H18" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, offline)</t>
+          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="I18" s="54" t="inlineStr">
         <is>
-          <t>• Frame an unfamiliar engineering problem as a machine learning task, unaided.
-• Prepare data and control leakage within a pipeline.
-• Build and compare at least two models under a single valid protocol.
-• Evaluate with a justified metric and report the result in engineering terms.
-• State the model's limitations and the conditions under which it should not be used.
-• Explain their own reasoning in writing without any tool.</t>
+          <t>• Split data by whole equipment groups and fit models on training rows only.
+• Compare a baseline, a straight line, a tree, a ridge curve and nearest neighbours on the same validation rows.
+• Count classification outcomes and work out a cost, and run cross-validation by group.
+• Test whether an extra input helps, and choose a model inside stated limits.
+• Explain the choices: sealed test rows, training-only fill values, scaling and the ridge penalty.</t>
         </is>
       </c>
       <c r="J18" s="54" t="inlineStr">
         <is>
-          <t>• 0:00-0:15  Seating, machine allocation, variant distribution, rules read aloud, offline mode confirmed.
-• 0:15-2:15  TEST, PART A (practical, 2 hours). Individual, unfamiliar dataset from the cohort's domain. Tasks: state the ML task and name the target; prepare the data with justified decisions; build at least two models inside a leak-proof pipeline; evaluate with a justified metric and validate properly; report the result in physical or operational units; state three limitations.
-• 2:15-2:40  TEST, PART B (written reasoning, 25 minutes, typed offline responses only; no code execution). Why this metric. Where could this pipeline leak. What would change your recommendation. Would you deploy this, and what would you require first.
-• 2:40-3:00  Collection, structural check, dismissal. Week 15 demo running order confirmed.</t>
+          <t>• 0:00-0:15  Entry page, notebook and CSV downloaded, rules read aloud, identity cell checked.
+• 0:15-2:15  CODING (120 minutes). Individual, in Colab. Eight functions covering Weeks 8 to 13, from group_split to ridge_and_knn. The notebook states the columns, return formats and marks.
+• 2:15-2:40  INTERPRETATION AND CHECKING (25 minutes). Six scenario choices recorded in DECISIONS, then Restart and Run all.
+• 2:40-3:00  FINAL SAVE AND SUBMISSION (20 minutes). Submit test button, generated form link, confirmation. Week 15 demo running order confirmed.</t>
         </is>
       </c>
       <c r="K18" s="54" t="inlineStr">
@@ -12893,14 +12890,14 @@
       </c>
       <c r="L18" s="54" t="inlineStr">
         <is>
-          <t>• Permitted: Python, VS Code or Jupyter, pandas, NumPy, matplotlib, seaborn, scikit-learn, and the offline documentation bundle.
-• Prohibited: internet, AI assistants, messaging. The room runs offline.
-• The offline bundle must include the scikit-learn API documentation - the test examines judgement, not memory of parameter names.</t>
+          <t>• Permitted: Colab, the submission form and any other resource the invigilator announces.
+• Prohibited: AI assistants, messaging and copied answers.
+• The notebook explains the columns and return formats, so the test examines judgement rather than memory of parameter names.</t>
         </is>
       </c>
       <c r="M18" s="54" t="inlineStr">
         <is>
-          <t>The test is the practical. Duration 2h00 practical + 0h25 written. Three parallel dataset variants in a checkerboard seating pattern.</t>
+          <t>The test is a coding practical in Colab, three hours from the start including setup, checking and submission. Three parallel dataset variants are issued by the entry page, and the deterministic grader re-runs the submitted code on other data.</t>
         </is>
       </c>
       <c r="N18" s="54" t="inlineStr">
@@ -12930,24 +12927,22 @@
       </c>
       <c r="S18" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 2 = 20% of the Semester 1 mark. Individual. Rubric: task framing 10, data preparation and leakage control 20, modelling protocol 20, evaluation and metric justification 20, engineering interpretation and limits 20, code clarity 10.</t>
+          <t>PRACTICAL TEST 2 = 20% of the Semester 1 mark. Individual. Rubric: group split 10, baseline, linear and tree predictions 15, MAE and RMSE 5, classification and cost 10, group cross-validation 10, feature ablation 10, model selection 10, ridge and nearest neighbours 15, six interpretation choices 15.</t>
         </is>
       </c>
       <c r="T18" s="54" t="inlineStr">
         <is>
-          <t>• Author three parallel dataset variants of matched difficulty, each with a model answer and a mark scheme.
-• Build and test the offline bundle, including scikit-learn documentation, on a machine with the network physically disconnected.
-• Confirm the capacity plan. Cohort A will very likely need two sittings; this must be timetabled with the Faculty by Week 7 at the latest.
-• Write the structural auto-check script (runs top to bottom, required sections present, no internet calls) to make large-cohort marking feasible.
-• Agree the moderation sample and the double-marking plan with the Faculty.
+          <t>• Author three parallel dataset variants of matched difficulty, each with a reference solution. The grader re-runs submitted code on unseen data.
+• Test the entry page, notebook download, Submit test button and form link with one account for each variant.
+• Confirm sittings, invigilators and Colab capacity with the Faculty. Cohort A is about 100 students.
+• Agree the moderation sample with the Faculty.
 • Prepare the Week 15 demo running order, two typed defence prompts and the digital submission check.</t>
         </is>
       </c>
       <c r="U18" s="54" t="inlineStr">
         <is>
-          <t>• Invigilated offline lab; confirmed machine count; spare machines; power contingency.
-• USB or local drop folder collection.
-• Printed task sheets per variant; Part B answers typed into the notebook.
+          <t>• A room with stable wifi and a Colab-capable laptop for every student; confirmed seat count; power contingency.
+• Entry links or QR codes for each variant.
 • Second invigilator for any sitting above 40 students.
 • Rubric published in Week 11.</t>
         </is>
@@ -13137,6 +13132,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="31.5" customHeight="1" s="36">
       <c r="A4" s="42" t="inlineStr">
         <is>
@@ -13367,12 +13363,12 @@
       </c>
       <c r="B11" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 1 - Data Investigation (individual, offline)</t>
+          <t>PRACTICAL TEST 1 - Data Investigation (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="C11" s="54" t="inlineStr">
         <is>
-          <t>Format, duration, rules, offline bundle, rubric, invigilation plan, auto-check script, moderation plan.</t>
+          <t>Format, duration, rules, issued notebook bundle, rubric, moderation plan.</t>
         </is>
       </c>
       <c r="D11" s="54" t="inlineStr">
@@ -13387,9 +13383,9 @@
       </c>
       <c r="F11" s="54" t="inlineStr">
         <is>
-          <t>[A] DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, offline bundle.
-[B] DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, offline bundle.
-[C] DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, offline bundle.</t>
+          <t>[A] DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, issued notebook bundle.
+[B] DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, issued notebook bundle.
+[C] DIVERGENT: the three dataset variants and their mark schemes. SHARED: format, rules, duration, rubric, issued notebook bundle.</t>
         </is>
       </c>
     </row>
@@ -13591,12 +13587,12 @@
       </c>
       <c r="B18" s="54" t="inlineStr">
         <is>
-          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, offline)</t>
+          <t>PRACTICAL TEST 2 - End-to-End Engineering Machine Learning (individual, timed Colab practical)</t>
         </is>
       </c>
       <c r="C18" s="54" t="inlineStr">
         <is>
-          <t>Format, duration, rules, offline bundle, rubric, invigilation, auto-check script, moderation.</t>
+          <t>Format, duration, rules, issued notebook bundle, rubric, moderation.</t>
         </is>
       </c>
       <c r="D18" s="54" t="inlineStr">
@@ -13649,6 +13645,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="45.75" customHeight="1" s="36">
       <c r="A21" s="56" t="inlineStr">
         <is>
@@ -13700,6 +13697,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="19.5" customHeight="1" s="36">
       <c r="A4" s="57" t="inlineStr">
         <is>
@@ -13842,7 +13840,7 @@
       </c>
       <c r="C9" s="47" t="inlineStr">
         <is>
-          <t>Individual, offline, 2h25</t>
+          <t>Individual, timed Colab, 3h</t>
         </is>
       </c>
       <c r="D9" s="58" t="n">
@@ -13850,12 +13848,12 @@
       </c>
       <c r="E9" s="47" t="inlineStr">
         <is>
-          <t>Investigation notebook + typed reasoning cells in the notebook. Part A answers are entered in a structured answers interface so 52 of the 100 marks are checked deterministically; the remaining 48 require validated written and visual evidence assessment before release.</t>
+          <t>Take-home Colab practical, 3 hours from the start. Eight coding tasks checked deterministically on other data with the same columns: reading and inspecting the file, charts before and after cleaning, cleaning, statistics, grouping, a function and a loop with conditions. No written report. AI assistance is not permitted.</t>
         </is>
       </c>
       <c r="F9" s="47" t="inlineStr">
         <is>
-          <t>Test 1 rubric (see Rubrics sheet). Current draft: 52 executed / 48 evidence marks; task-specific checks and calibration required.</t>
+          <t>Test 1 rubric (see Rubrics sheet). Eight coded tasks, 100 marks, all checked deterministically on other data.</t>
         </is>
       </c>
     </row>
@@ -13872,7 +13870,7 @@
       </c>
       <c r="C10" s="47" t="inlineStr">
         <is>
-          <t>Individual, offline, 2h25</t>
+          <t>Individual, timed Colab, 3h</t>
         </is>
       </c>
       <c r="D10" s="58" t="n">
@@ -13880,12 +13878,12 @@
       </c>
       <c r="E10" s="47" t="inlineStr">
         <is>
-          <t>End-to-end notebook + typed reasoning cells in the notebook. Current executed contracts supply 30 marks of the 100; the remaining 70 require validated evidence and local rubric assessment before release.</t>
+          <t>Colab practical, 180 minutes, covering Weeks 8 to 13. Eight coding tasks (group split 10, baseline, linear and tree predictions 15, MAE and RMSE 5, classification and cost 10, group cross-validation 10, feature ablation 10, model selection 10, ridge and nearest neighbours 15) re-run by the lecturer's grader on unseen data, plus six interpretation choices (15). No separate written report. AI assistance is not permitted.</t>
         </is>
       </c>
       <c r="F10" s="47" t="inlineStr">
         <is>
-          <t>Test 2 rubric (see Rubrics sheet). Current draft: 30 executed / 70 evidence marks; task-specific checks and calibration required.</t>
+          <t>Test 2 rubric (see Rubrics sheet). Eight coded functions (85 marks) and six interpretation choices (15 marks), checked deterministically.</t>
         </is>
       </c>
     </row>
@@ -14022,6 +14020,8 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
+    <row r="18"/>
     <row r="19" ht="19.5" customHeight="1" s="36">
       <c r="A19" s="57" t="inlineStr">
         <is>
@@ -14278,6 +14278,8 @@
       <c r="E30" s="60" t="n"/>
       <c r="F30" s="60" t="n"/>
     </row>
+    <row r="31"/>
+    <row r="32"/>
     <row r="33" ht="19.5" customHeight="1" s="36">
       <c r="A33" s="57" t="inlineStr">
         <is>
@@ -14300,12 +14302,12 @@
     <row r="35" ht="51.75" customHeight="1" s="36">
       <c r="A35" s="40" t="inlineStr">
         <is>
-          <t>Why the tests run offline</t>
+          <t>Why the tests are unaided</t>
         </is>
       </c>
       <c r="B35" s="41" t="inlineStr">
         <is>
-          <t>An invigilated lab and approved-materials rules support the unaided assessment. Offline access alone does not block a local AI model. AI assistance is permitted and actively taught in coursework, where students explain and defend their work; it is excluded from the two tests, which certify unaided capability. Students are told the reasoning in Week 6, not on the day.</t>
+          <t>Approved-materials rules, hidden-data grading and an understanding check support the unaided assessment. No setting in Colab blocks an AI assistant. AI assistance is permitted and actively taught in coursework, where students explain and defend their work; it is excluded from the two tests, which certify unaided capability. Students are told the reasoning in Week 6, not on the day.</t>
         </is>
       </c>
     </row>
@@ -14397,7 +14399,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D60"/>
+  <dimension ref="A1:E65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="34" customWidth="1" style="35" min="1" max="1"/>
@@ -14420,6 +14422,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="19.5" customHeight="1" s="36">
       <c r="A4" s="57" t="inlineStr">
         <is>
@@ -14574,6 +14577,7 @@
       <c r="C13" s="60" t="n"/>
       <c r="D13" s="60" t="n"/>
     </row>
+    <row r="14"/>
     <row r="15" ht="19.5" customHeight="1" s="36">
       <c r="A15" s="57" t="inlineStr">
         <is>
@@ -14606,15 +14610,15 @@
     <row r="17" ht="43.5" customHeight="1" s="36">
       <c r="A17" s="46" t="inlineStr">
         <is>
-          <t>Loading &amp; profiling</t>
+          <t>Read and inspect the raw data</t>
         </is>
       </c>
       <c r="B17" s="65" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C17" s="47" t="inlineStr">
         <is>
-          <t>Data loaded correctly; shape, types and summary produced; the dataset is described accurately in the student's own words.</t>
+          <t>Read the CSV with pandas into raw_data without changing it. Show the first and last rows, shape, row count, column type, info(), describe(), missing counts per column, the repeated record_id count and the invalid records.</t>
         </is>
       </c>
       <c r="D17" s="47" t="n"/>
@@ -14622,15 +14626,15 @@
     <row r="18" ht="43.5" customHeight="1" s="36">
       <c r="A18" s="46" t="inlineStr">
         <is>
-          <t>Cleaning decisions &amp; justification</t>
+          <t>Visualisation before cleaning</t>
         </is>
       </c>
       <c r="B18" s="65" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C18" s="47" t="inlineStr">
         <is>
-          <t>Defects found. Each handling decision stated AND justified. Marks are for the justification - an unjustified correct fix scores roughly half.</t>
+          <t>Scatter chart of load_pct against target from the raw data: correct points 4, title 2, horizontal label with % 2, vertical label with unit 2.</t>
         </is>
       </c>
       <c r="D18" s="47" t="n"/>
@@ -14638,7 +14642,7 @@
     <row r="19" ht="43.5" customHeight="1" s="36">
       <c r="A19" s="46" t="inlineStr">
         <is>
-          <t>Visualisation</t>
+          <t>Clean the data</t>
         </is>
       </c>
       <c r="B19" s="65" t="n">
@@ -14646,7 +14650,7 @@
       </c>
       <c r="C19" s="47" t="inlineStr">
         <is>
-          <t>Three charts, each captioned with the question it answers. Correct chart type. Axes labelled with units. No decoration without purpose.</t>
+          <t>Keep the first row per record_id, remove rows with missing target or load_pct outside 0 to 100, fill missing ambient_c with the median of the retained rows. 4 marks for each correctly cleaned column.</t>
         </is>
       </c>
       <c r="D19" s="47" t="n"/>
@@ -14654,15 +14658,15 @@
     <row r="20" ht="43.5" customHeight="1" s="36">
       <c r="A20" s="46" t="inlineStr">
         <is>
-          <t>Findings</t>
+          <t>Visualisation after cleaning</t>
         </is>
       </c>
       <c r="B20" s="65" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C20" s="47" t="inlineStr">
         <is>
-          <t>Five findings, supported by evidence from the data, stated with correct magnitudes and units. A wrong number loses the mark even if the method was right.</t>
+          <t>The same chart from the cleaned data, with the same four marking parts. No written comparison is required.</t>
         </is>
       </c>
       <c r="D20" s="47" t="n"/>
@@ -14670,7 +14674,7 @@
     <row r="21" ht="43.5" customHeight="1" s="36">
       <c r="A21" s="46" t="inlineStr">
         <is>
-          <t>Engineering interpretation</t>
+          <t>Calculate statistics</t>
         </is>
       </c>
       <c r="B21" s="65" t="n">
@@ -14678,7 +14682,7 @@
       </c>
       <c r="C21" s="47" t="inlineStr">
         <is>
-          <t>One recommendation that an engineer could act on, plus a clear statement of what further data would be needed.</t>
+          <t>Mean, sum, median, count and sample standard deviation of target, and every most frequent equipment_id. Six answers at 2.5 marks each.</t>
         </is>
       </c>
       <c r="D21" s="47" t="n"/>
@@ -14686,7 +14690,7 @@
     <row r="22" ht="43.5" customHeight="1" s="36">
       <c r="A22" s="46" t="inlineStr">
         <is>
-          <t>Clarity &amp; reproducibility</t>
+          <t>Group and aggregate</t>
         </is>
       </c>
       <c r="B22" s="65" t="n">
@@ -14694,97 +14698,98 @@
       </c>
       <c r="C22" s="47" t="inlineStr">
         <is>
-          <t>Notebook runs top to bottom. Logical order. Markdown explains intent. No dead code.</t>
+          <t>equipment_summary built with groupby and agg: mean and count of target for each equipment, 5 marks per column.</t>
         </is>
       </c>
       <c r="D22" s="47" t="n"/>
     </row>
-    <row r="23" ht="18" customHeight="1" s="36">
-      <c r="A23" s="59" t="inlineStr">
+    <row r="23" ht="43.5" customHeight="1" s="36">
+      <c r="A23" s="46" t="inlineStr">
+        <is>
+          <t>Reuse your statistics in one function</t>
+        </is>
+      </c>
+      <c r="B23" s="65" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" s="47" t="inlineStr">
+        <is>
+          <t>A function that returns the mean, sum and median of any column of any table, checked on other numbers.</t>
+        </is>
+      </c>
+      <c r="D23" s="47" t="n"/>
+    </row>
+    <row r="24" ht="43.5" customHeight="1" s="36">
+      <c r="A24" s="46" t="inlineStr">
+        <is>
+          <t>Conditions and a loop</t>
+        </is>
+      </c>
+      <c r="B24" s="65" t="n">
+        <v>10</v>
+      </c>
+      <c r="C24" s="47" t="inlineStr">
+        <is>
+          <t>A for loop with if, elif and else counting loads as low (below 40), medium (40 to 75) or high (above 75): correct counts 6, loop 2, conditions 2.</t>
+        </is>
+      </c>
+      <c r="D24" s="47" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="36">
+      <c r="A25" s="59" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="59">
-        <f>SUM(B17:B22)</f>
+      <c r="B25" s="59">
+        <f>SUM(B17:B24)</f>
         <v/>
       </c>
-      <c r="C23" s="60" t="n"/>
-      <c r="D23" s="60" t="n"/>
-    </row>
-    <row r="25" ht="19.5" customHeight="1" s="36">
-      <c r="A25" s="57" t="inlineStr">
+      <c r="C25" s="60" t="n"/>
+      <c r="D25" s="60" t="n"/>
+    </row>
+    <row r="26" ht="21.75" customHeight="1" s="36"/>
+    <row r="27" ht="19.5" customHeight="1" s="36">
+      <c r="A27" s="57" t="inlineStr">
         <is>
           <t>Practical Test 2 - End-to-End Engineering ML (20%)</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="21.75" customHeight="1" s="36">
-      <c r="A26" s="42" t="inlineStr">
+    <row r="28" ht="21.75" customHeight="1" s="36">
+      <c r="A28" s="42" t="inlineStr">
         <is>
           <t>Criterion</t>
         </is>
       </c>
-      <c r="B26" s="42" t="inlineStr">
+      <c r="B28" s="42" t="inlineStr">
         <is>
           <t>Marks</t>
         </is>
       </c>
-      <c r="C26" s="42" t="inlineStr">
+      <c r="C28" s="42" t="inlineStr">
         <is>
           <t>What earns the marks</t>
         </is>
       </c>
-      <c r="D26" s="42" t="inlineStr">
+      <c r="D28" s="42" t="inlineStr">
         <is>
           <t>Marker note</t>
         </is>
       </c>
-    </row>
-    <row r="27" ht="43.5" customHeight="1" s="36">
-      <c r="A27" s="46" t="inlineStr">
-        <is>
-          <t>Task framing</t>
-        </is>
-      </c>
-      <c r="B27" s="65" t="n">
-        <v>10</v>
-      </c>
-      <c r="C27" s="47" t="inlineStr">
-        <is>
-          <t>The ML task is correctly identified, the target named, and regression vs classification correctly chosen and justified.</t>
-        </is>
-      </c>
-      <c r="D27" s="47" t="n"/>
-    </row>
-    <row r="28" ht="43.5" customHeight="1" s="36">
-      <c r="A28" s="46" t="inlineStr">
-        <is>
-          <t>Data preparation &amp; leakage control</t>
-        </is>
-      </c>
-      <c r="B28" s="65" t="n">
-        <v>20</v>
-      </c>
-      <c r="C28" s="47" t="inlineStr">
-        <is>
-          <t>Cleaning and encoding appropriate. Split made before any fitting. Pipeline used. No leakage present - a leak found by the marker caps this criterion at zero.</t>
-        </is>
-      </c>
-      <c r="D28" s="47" t="n"/>
     </row>
     <row r="29" ht="43.5" customHeight="1" s="36">
       <c r="A29" s="46" t="inlineStr">
         <is>
-          <t>Modelling protocol</t>
+          <t>Equipment-group split</t>
         </is>
       </c>
       <c r="B29" s="65" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C29" s="47" t="inlineStr">
         <is>
-          <t>At least two models built and compared under identical conditions. Baseline included. Hyperparameters handled sensibly.</t>
+          <t>group_split returns the train (E1 to E4), validation (E5) and test (E6) record_id lists in input order, without using target values. Week 10.</t>
         </is>
       </c>
       <c r="D29" s="47" t="n"/>
@@ -14792,15 +14797,15 @@
     <row r="30" ht="43.5" customHeight="1" s="36">
       <c r="A30" s="46" t="inlineStr">
         <is>
-          <t>Evaluation &amp; metric justification</t>
+          <t>Baseline, linear and tree predictions</t>
         </is>
       </c>
       <c r="B30" s="65" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C30" s="47" t="inlineStr">
         <is>
-          <t>Correct metrics computed. Metric choice defended against the cost of error. Cross-validation reported with a spread, not a single number.</t>
+          <t>predict_regression fits a training-mean baseline, linear regression and a decision tree (max_depth 4, random_state 17) on load_pct and ambient_c, fits preprocessing on training rows only, and returns three prediction lists. Week 8.</t>
         </is>
       </c>
       <c r="D30" s="47" t="n"/>
@@ -14808,15 +14813,15 @@
     <row r="31" ht="43.5" customHeight="1" s="36">
       <c r="A31" s="46" t="inlineStr">
         <is>
-          <t>Engineering interpretation &amp; limits</t>
+          <t>MAE and RMSE</t>
         </is>
       </c>
       <c r="B31" s="65" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="C31" s="47" t="inlineStr">
         <is>
-          <t>The result is stated in physical or operational units. Three genuine limitations given. A clear position on whether it should be deployed.</t>
+          <t>regression_errors returns mae and rmse over the same paired observations, unrounded. Week 8.</t>
         </is>
       </c>
       <c r="D31" s="47" t="n"/>
@@ -14824,7 +14829,7 @@
     <row r="32" ht="43.5" customHeight="1" s="36">
       <c r="A32" s="46" t="inlineStr">
         <is>
-          <t>Code clarity</t>
+          <t>Classification and cost</t>
         </is>
       </c>
       <c r="B32" s="65" t="n">
@@ -14832,360 +14837,444 @@
       </c>
       <c r="C32" s="47" t="inlineStr">
         <is>
-          <t>Runs top to bottom. Readable. Commented where the intent is not obvious.</t>
+          <t>classification_metrics returns tp, tn, fp, fn, precision, recall and cost (5 per missed warning plus 1 per false alarm), with zero for an undefined ratio. Week 9.</t>
         </is>
       </c>
       <c r="D32" s="47" t="n"/>
     </row>
-    <row r="33" ht="18" customHeight="1" s="36">
-      <c r="A33" s="59" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B33" s="59">
-        <f>SUM(B27:B32)</f>
-        <v/>
-      </c>
-      <c r="C33" s="60" t="n"/>
-      <c r="D33" s="60" t="n"/>
-    </row>
-    <row r="35" ht="19.5" customHeight="1" s="36">
-      <c r="A35" s="57" t="inlineStr">
-        <is>
-          <t>Data Analysis Project (10%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="21.75" customHeight="1" s="36">
-      <c r="A36" s="42" t="inlineStr">
-        <is>
-          <t>Criterion</t>
-        </is>
-      </c>
-      <c r="B36" s="42" t="inlineStr">
-        <is>
-          <t>Marks</t>
-        </is>
-      </c>
-      <c r="C36" s="42" t="inlineStr">
-        <is>
-          <t>What earns the marks</t>
-        </is>
-      </c>
-      <c r="D36" s="42" t="inlineStr">
-        <is>
-          <t>Marker note</t>
-        </is>
-      </c>
+    <row r="33" ht="43.5" customHeight="1" s="36">
+      <c r="A33" s="46" t="inlineStr">
+        <is>
+          <t>Group cross-validation</t>
+        </is>
+      </c>
+      <c r="B33" s="65" t="n">
+        <v>10</v>
+      </c>
+      <c r="C33" s="47" t="inlineStr">
+        <is>
+          <t>group_cv_mae holds out E1 to E5 in turn, fits a straight line on the other four groups and returns the five fold MAEs, their mean and their sample standard deviation. E6 is never used. Week 10.</t>
+        </is>
+      </c>
+      <c r="D33" s="47" t="n"/>
+    </row>
+    <row r="34" ht="43.5" customHeight="1" s="36">
+      <c r="A34" s="46" t="inlineStr">
+        <is>
+          <t>Feature ablation</t>
+        </is>
+      </c>
+      <c r="B34" s="65" t="n">
+        <v>10</v>
+      </c>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>ablation_metrics compares a straight line on load_pct and ambient_c with one that adds load_pct times ambient_c, on the same validation records, and returns both MAEs and the improvement. Week 11.</t>
+        </is>
+      </c>
+      <c r="D34" s="47" t="n"/>
+    </row>
+    <row r="35" ht="43.5" customHeight="1" s="36">
+      <c r="A35" s="46" t="inlineStr">
+        <is>
+          <t>Model selection</t>
+        </is>
+      </c>
+      <c r="B35" s="65" t="n">
+        <v>10</v>
+      </c>
+      <c r="C35" s="47" t="inlineStr">
+        <is>
+          <t>select_model keeps the candidates that meet the MAE and latency limits and picks the smallest validation MAE, then the smaller latency, then the name. Week 12.</t>
+        </is>
+      </c>
+      <c r="D35" s="47" t="n"/>
+    </row>
+    <row r="36" ht="43.5" customHeight="1" s="36">
+      <c r="A36" s="46" t="inlineStr">
+        <is>
+          <t>Ridge and nearest neighbours</t>
+        </is>
+      </c>
+      <c r="B36" s="65" t="n">
+        <v>15</v>
+      </c>
+      <c r="C36" s="47" t="inlineStr">
+        <is>
+          <t>ridge_and_knn fits a degree-3 ridge curve on load_pct (alpha 1) and a 3-neighbour model on scaled load_pct and ambient_c, using training rows only, and returns both validation MAEs and which is better. Week 13.</t>
+        </is>
+      </c>
+      <c r="D36" s="47" t="n"/>
     </row>
     <row r="37" ht="43.5" customHeight="1" s="36">
       <c r="A37" s="46" t="inlineStr">
         <is>
+          <t>Structured interpretation</t>
+        </is>
+      </c>
+      <c r="B37" s="65" t="n">
+        <v>15</v>
+      </c>
+      <c r="C37" s="47" t="inlineStr">
+        <is>
+          <t>Six scenario choices (A, B or C) on whole-group splits, training-only fill values, cost and threshold, the sealed test rows, choosing a ridge penalty and scaling for nearest neighbours. 2.5 marks each.</t>
+        </is>
+      </c>
+      <c r="D37" s="47" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="36">
+      <c r="A38" s="59" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B38" s="59">
+        <f>SUM(B29:B37)</f>
+        <v/>
+      </c>
+      <c r="C38" s="60" t="n"/>
+      <c r="D38" s="60" t="n"/>
+    </row>
+    <row r="39" ht="21.75" customHeight="1" s="36"/>
+    <row r="40" ht="19.5" customHeight="1" s="36">
+      <c r="A40" s="57" t="inlineStr">
+        <is>
+          <t>Data Analysis Project (10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="21.75" customHeight="1" s="36">
+      <c r="A41" s="42" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B41" s="42" t="inlineStr">
+        <is>
+          <t>Marks</t>
+        </is>
+      </c>
+      <c r="C41" s="42" t="inlineStr">
+        <is>
+          <t>What earns the marks</t>
+        </is>
+      </c>
+      <c r="D41" s="42" t="inlineStr">
+        <is>
+          <t>Marker note</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="43.5" customHeight="1" s="36">
+      <c r="A42" s="46" t="inlineStr">
+        <is>
           <t>Question &amp; dataset fit</t>
         </is>
       </c>
-      <c r="B37" s="65" t="n">
+      <c r="B42" s="65" t="n">
         <v>20</v>
       </c>
-      <c r="C37" s="47" t="inlineStr">
+      <c r="C42" s="47" t="inlineStr">
         <is>
           <t>A real engineering question is stated, and the chosen dataset can actually answer it. Provenance and licence stated.</t>
         </is>
       </c>
-      <c r="D37" s="47" t="n"/>
-    </row>
-    <row r="38" ht="43.5" customHeight="1" s="36">
-      <c r="A38" s="46" t="inlineStr">
+      <c r="D42" s="47" t="n"/>
+    </row>
+    <row r="43" ht="43.5" customHeight="1" s="36">
+      <c r="A43" s="46" t="inlineStr">
         <is>
           <t>Data quality work</t>
         </is>
       </c>
-      <c r="B38" s="65" t="n">
+      <c r="B43" s="65" t="n">
         <v>25</v>
       </c>
-      <c r="C38" s="47" t="inlineStr">
+      <c r="C43" s="47" t="inlineStr">
         <is>
           <t>Defects found and handled with written justification. A data quality statement is present.</t>
         </is>
       </c>
-      <c r="D38" s="47" t="n"/>
-    </row>
-    <row r="39" ht="43.5" customHeight="1" s="36">
-      <c r="A39" s="46" t="inlineStr">
+      <c r="D43" s="47" t="n"/>
+    </row>
+    <row r="44" ht="43.5" customHeight="1" s="36">
+      <c r="A44" s="46" t="inlineStr">
         <is>
           <t>Analysis &amp; visualisation</t>
         </is>
       </c>
-      <c r="B39" s="65" t="n">
+      <c r="B44" s="65" t="n">
         <v>30</v>
       </c>
-      <c r="C39" s="47" t="inlineStr">
+      <c r="C44" s="47" t="inlineStr">
         <is>
           <t>Four or more charts, each answering a stated question. Correct chart types, labelled axes, findings in the captions.</t>
         </is>
       </c>
-      <c r="D39" s="47" t="n"/>
-    </row>
-    <row r="40" ht="43.5" customHeight="1" s="36">
-      <c r="A40" s="46" t="inlineStr">
+      <c r="D44" s="47" t="n"/>
+    </row>
+    <row r="45" ht="43.5" customHeight="1" s="36">
+      <c r="A45" s="46" t="inlineStr">
         <is>
           <t>Findings &amp; interpretation</t>
         </is>
       </c>
-      <c r="B40" s="65" t="n">
+      <c r="B45" s="65" t="n">
         <v>20</v>
       </c>
-      <c r="C40" s="47" t="inlineStr">
+      <c r="C45" s="47" t="inlineStr">
         <is>
           <t>Conclusions supported by the analysis, stated in engineering terms, with limitations acknowledged.</t>
         </is>
       </c>
-      <c r="D40" s="47" t="n"/>
-    </row>
-    <row r="41" ht="43.5" customHeight="1" s="36">
-      <c r="A41" s="46" t="inlineStr">
-        <is>
-          <t>Individual contribution log</t>
-        </is>
-      </c>
-      <c r="B41" s="65" t="n">
-        <v>5</v>
-      </c>
-      <c r="C41" s="47" t="inlineStr">
-        <is>
-          <t>Present, specific, and consistent with the repository's commit history.</t>
-        </is>
-      </c>
-      <c r="D41" s="47" t="n"/>
-    </row>
-    <row r="42" ht="18" customHeight="1" s="36">
-      <c r="A42" s="59" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B42" s="59">
-        <f>SUM(B37:B41)</f>
-        <v/>
-      </c>
-      <c r="C42" s="60" t="n"/>
-      <c r="D42" s="60" t="n"/>
-    </row>
-    <row r="44" ht="19.5" customHeight="1" s="36">
-      <c r="A44" s="57" t="inlineStr">
-        <is>
-          <t>Weekly quizzes (10%) - how the five questions in each are marked</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="21.75" customHeight="1" s="36">
-      <c r="A45" s="42" t="inlineStr">
-        <is>
-          <t>Criterion</t>
-        </is>
-      </c>
-      <c r="B45" s="42" t="inlineStr">
-        <is>
-          <t>Marks</t>
-        </is>
-      </c>
-      <c r="C45" s="42" t="inlineStr">
-        <is>
-          <t>What earns the marks</t>
-        </is>
-      </c>
-      <c r="D45" s="42" t="inlineStr">
-        <is>
-          <t>Marker note</t>
-        </is>
-      </c>
+      <c r="D45" s="47" t="n"/>
     </row>
     <row r="46" ht="43.5" customHeight="1" s="36">
       <c r="A46" s="46" t="inlineStr">
         <is>
+          <t>Individual contribution log</t>
+        </is>
+      </c>
+      <c r="B46" s="65" t="n">
+        <v>5</v>
+      </c>
+      <c r="C46" s="47" t="inlineStr">
+        <is>
+          <t>Present, specific, and consistent with the repository's commit history.</t>
+        </is>
+      </c>
+      <c r="D46" s="47" t="n"/>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="36">
+      <c r="A47" s="59" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B47" s="59">
+        <f>SUM(B42:B46)</f>
+        <v/>
+      </c>
+      <c r="C47" s="60" t="n"/>
+      <c r="D47" s="60" t="n"/>
+    </row>
+    <row r="48" s="36"/>
+    <row r="49" ht="19.5" customHeight="1" s="36">
+      <c r="A49" s="57" t="inlineStr">
+        <is>
+          <t>Weekly quizzes (10%) - how the five questions in each are marked</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="21.75" customHeight="1" s="36">
+      <c r="A50" s="42" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B50" s="42" t="inlineStr">
+        <is>
+          <t>Marks</t>
+        </is>
+      </c>
+      <c r="C50" s="42" t="inlineStr">
+        <is>
+          <t>What earns the marks</t>
+        </is>
+      </c>
+      <c r="D50" s="42" t="inlineStr">
+        <is>
+          <t>Marker note</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="43.5" customHeight="1" s="36">
+      <c r="A51" s="46" t="inlineStr">
+        <is>
           <t>Diagnosis of a silent wrong answer</t>
         </is>
       </c>
-      <c r="B46" s="65" t="n">
+      <c r="B51" s="65" t="n">
         <v>40</v>
       </c>
-      <c r="C46" s="47" t="inlineStr">
+      <c r="C51" s="47" t="inlineStr">
         <is>
           <t>Two of the five questions show code that runs cleanly and returns a wrong result. The student must name the cause. Auto-marked, single correct option, distractors chosen to be the plausible wrong diagnoses.</t>
         </is>
       </c>
-      <c r="D46" s="47" t="n"/>
-    </row>
-    <row r="47" ht="43.5" customHeight="1" s="36">
-      <c r="A47" s="46" t="inlineStr">
+      <c r="D51" s="47" t="n"/>
+    </row>
+    <row r="52" ht="43.5" customHeight="1" s="36">
+      <c r="A52" s="46" t="inlineStr">
         <is>
           <t>Reading an error or a traceback</t>
         </is>
       </c>
-      <c r="B47" s="65" t="n">
+      <c r="B52" s="65" t="n">
         <v>20</v>
       </c>
-      <c r="C47" s="47" t="inlineStr">
+      <c r="C52" s="47" t="inlineStr">
         <is>
           <t>One question shows a traceback or a failing cell. The student identifies the offending line or the cause. Auto-marked.</t>
         </is>
       </c>
-      <c r="D47" s="47" t="n"/>
-    </row>
-    <row r="48" ht="43.5" customHeight="1" s="36">
-      <c r="A48" s="46" t="inlineStr">
+      <c r="D52" s="47" t="n"/>
+    </row>
+    <row r="53" ht="43.5" customHeight="1" s="36">
+      <c r="A53" s="46" t="inlineStr">
         <is>
           <t>Interpreting an output, chart or table</t>
         </is>
       </c>
-      <c r="B48" s="65" t="n">
+      <c r="B53" s="65" t="n">
         <v>20</v>
       </c>
-      <c r="C48" s="47" t="inlineStr">
+      <c r="C53" s="47" t="inlineStr">
         <is>
           <t>One question supplies a real output - a describe(), a confusion matrix, an ablation table - and asks what it means for the engineering problem. Auto-marked.</t>
         </is>
       </c>
-      <c r="D48" s="47" t="n"/>
-    </row>
-    <row r="49" ht="43.5" customHeight="1" s="36">
-      <c r="A49" s="46" t="inlineStr">
-        <is>
-          <t>Judgement under a stated constraint</t>
-        </is>
-      </c>
-      <c r="B49" s="65" t="n">
-        <v>20</v>
-      </c>
-      <c r="C49" s="47" t="inlineStr">
-        <is>
-          <t>One question gives a constraint (a cost, a false-alarm budget, a regulator) and asks which choice follows. Auto-marked, but the distractors are all defensible in the absence of the constraint, so the constraint has to be read.</t>
-        </is>
-      </c>
-      <c r="D49" s="47" t="n"/>
-    </row>
-    <row r="50" ht="18" customHeight="1" s="36">
-      <c r="A50" s="59" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B50" s="59">
-        <f>SUM(B46:B49)</f>
-        <v/>
-      </c>
-      <c r="C50" s="60" t="n"/>
-      <c r="D50" s="60" t="n"/>
-    </row>
-    <row r="52" ht="19.5" customHeight="1" s="36">
-      <c r="A52" s="57" t="inlineStr">
-        <is>
-          <t>Demo, viva &amp; individual reflection (10%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="21.75" customHeight="1" s="36">
-      <c r="A53" s="42" t="inlineStr">
-        <is>
-          <t>Criterion</t>
-        </is>
-      </c>
-      <c r="B53" s="42" t="inlineStr">
-        <is>
-          <t>Marks</t>
-        </is>
-      </c>
-      <c r="C53" s="42" t="inlineStr">
-        <is>
-          <t>What earns the marks</t>
-        </is>
-      </c>
-      <c r="D53" s="42" t="inlineStr">
-        <is>
-          <t>Marker note</t>
-        </is>
-      </c>
+      <c r="D53" s="47" t="n"/>
     </row>
     <row r="54" ht="43.5" customHeight="1" s="36">
       <c r="A54" s="46" t="inlineStr">
         <is>
+          <t>Judgement under a stated constraint</t>
+        </is>
+      </c>
+      <c r="B54" s="65" t="n">
+        <v>20</v>
+      </c>
+      <c r="C54" s="47" t="inlineStr">
+        <is>
+          <t>One question gives a constraint (a cost, a false-alarm budget, a regulator) and asks which choice follows. Auto-marked, but the distractors are all defensible in the absence of the constraint, so the constraint has to be read.</t>
+        </is>
+      </c>
+      <c r="D54" s="47" t="n"/>
+    </row>
+    <row r="55" ht="18" customHeight="1" s="36">
+      <c r="A55" s="59" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B55" s="59">
+        <f>SUM(B51:B54)</f>
+        <v/>
+      </c>
+      <c r="C55" s="60" t="n"/>
+      <c r="D55" s="60" t="n"/>
+    </row>
+    <row r="56" s="36"/>
+    <row r="57" ht="19.5" customHeight="1" s="36">
+      <c r="A57" s="57" t="inlineStr">
+        <is>
+          <t>Demo, viva &amp; individual reflection (10%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="21.75" customHeight="1" s="36">
+      <c r="A58" s="42" t="inlineStr">
+        <is>
+          <t>Criterion</t>
+        </is>
+      </c>
+      <c r="B58" s="42" t="inlineStr">
+        <is>
+          <t>Marks</t>
+        </is>
+      </c>
+      <c r="C58" s="42" t="inlineStr">
+        <is>
+          <t>What earns the marks</t>
+        </is>
+      </c>
+      <c r="D58" s="42" t="inlineStr">
+        <is>
+          <t>Marker note</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="43.5" customHeight="1" s="36">
+      <c r="A59" s="46" t="inlineStr">
+        <is>
           <t>Presentation evidence</t>
         </is>
       </c>
-      <c r="B54" s="65" t="n">
+      <c r="B59" s="65" t="n">
         <v>35</v>
       </c>
-      <c r="C54" s="47" t="inlineStr">
+      <c r="C59" s="47" t="inlineStr">
         <is>
           <t>Slides and narration notes explain the question, method, evidence and limitations for an engineering audience. The local text grader does not assess visual styling or spoken delivery.</t>
         </is>
       </c>
-      <c r="D54" s="47" t="n"/>
-    </row>
-    <row r="55" ht="43.5" customHeight="1" s="36">
-      <c r="A55" s="46" t="inlineStr">
+      <c r="D59" s="47" t="n"/>
+    </row>
+    <row r="60" ht="43.5" customHeight="1" s="36">
+      <c r="A60" s="46" t="inlineStr">
         <is>
           <t>Individual written defence</t>
         </is>
       </c>
-      <c r="B55" s="65" t="n">
+      <c r="B60" s="65" t="n">
         <v>40</v>
       </c>
-      <c r="C55" s="47" t="inlineStr">
+      <c r="C60" s="47" t="inlineStr">
         <is>
           <t>Two typed answers about the student's own repository identify specific cells/results and explain the decisions. Credit is based on the submitted evidence; live questioning is formative.</t>
         </is>
       </c>
-      <c r="D55" s="47" t="n"/>
-    </row>
-    <row r="56" ht="43.5" customHeight="1" s="36">
-      <c r="A56" s="46" t="inlineStr">
+      <c r="D60" s="47" t="n"/>
+    </row>
+    <row r="61" ht="43.5" customHeight="1" s="36">
+      <c r="A61" s="46" t="inlineStr">
         <is>
           <t>Reflection</t>
         </is>
       </c>
-      <c r="B56" s="65" t="n">
+      <c r="B61" s="65" t="n">
         <v>20</v>
       </c>
-      <c r="C56" s="47" t="inlineStr">
+      <c r="C61" s="47" t="inlineStr">
         <is>
           <t>500 words. Specific about what changed since Week 1, what remains difficult, and two concrete Semester 2 goals. Generic reflection scores low.</t>
         </is>
       </c>
-      <c r="D56" s="47" t="n"/>
-    </row>
-    <row r="57" ht="43.5" customHeight="1" s="36">
-      <c r="A57" s="46" t="inlineStr">
+      <c r="D61" s="47" t="n"/>
+    </row>
+    <row r="62" ht="43.5" customHeight="1" s="36">
+      <c r="A62" s="46" t="inlineStr">
         <is>
           <t>AI-use declaration</t>
         </is>
       </c>
-      <c r="B57" s="65" t="n">
+      <c r="B62" s="65" t="n">
         <v>5</v>
       </c>
-      <c r="C57" s="47" t="inlineStr">
+      <c r="C62" s="47" t="inlineStr">
         <is>
           <t>Present, complete and plausible against the repository history.</t>
         </is>
       </c>
-      <c r="D57" s="47" t="n"/>
-    </row>
-    <row r="58" ht="18" customHeight="1" s="36">
-      <c r="A58" s="59" t="inlineStr">
+      <c r="D62" s="47" t="n"/>
+    </row>
+    <row r="63" ht="18" customHeight="1" s="36">
+      <c r="A63" s="59" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B58" s="59">
-        <f>SUM(B54:B57)</f>
+      <c r="B63" s="59">
+        <f>SUM(B59:B62)</f>
         <v/>
       </c>
-      <c r="C58" s="60" t="n"/>
-      <c r="D58" s="60" t="n"/>
-    </row>
-    <row r="60" ht="48" customHeight="1" s="36">
-      <c r="A60" s="45" t="inlineStr">
+      <c r="C63" s="60" t="n"/>
+      <c r="D63" s="60" t="n"/>
+    </row>
+    <row r="64" s="36"/>
+    <row r="65" ht="48" customHeight="1" s="36">
+      <c r="A65" s="45" t="inlineStr">
         <is>
           <t>Apply the published execution, evidence and explanation criteria. Missing justification affects its specified criterion; there is no additional whole-submission penalty based on a live answer. Individual typed defence and reflection are separate from shared project marks. Live and peer feedback are formative.</t>
         </is>
@@ -15194,14 +15283,14 @@
   </sheetData>
   <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="A40:D40"/>
+    <mergeCell ref="A27:D27"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A52:D52"/>
     <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A65:D65"/>
+    <mergeCell ref="A57:D57"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A60:D60"/>
-    <mergeCell ref="A44:D44"/>
+    <mergeCell ref="A49:D49"/>
   </mergeCells>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>